<commit_message>
Daily MA Dashboard - 13-07-2026
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01274V9sTQVSgXqnFWW5yXaM
</commit_message>
<xml_diff>
--- a/outputs/daily_ma_dashboard.xlsx
+++ b/outputs/daily_ma_dashboard.xlsx
@@ -3298,9 +3298,9 @@
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="39" t="inlineStr">
         <is>
-          <t>1. JRTS สะสม -196,835.39 บาท เป็นต้นทุนแรงงานหลักที่ฉุด MA ลง แต่ยังคงดีกว่า Target (-242,738.65 บาท) อยู่ 45,903.26 บาท
-2. Association Product, Association Refer, Reciprocation ยังไม่มี Actual เลยตลอด 13 วันที่ผ่านมา (0 บาททั้ง 3 ช่องทาง)
-3. Shop Online (1+2) สะสม 3,722.04 บาท ดีกว่า Target 142.31 บาท อย่างมีนัยสำคัญ (+2,516%)</t>
+          <t>1. JRTS สะสม (14 วันแรก) -196,835.39 บาท ดีกว่า Target -242,738.65 บาท อยู่ 45,903.26 บาท เป็นตัวหลักที่ดึง %MA ให้ดีกว่าเป้า
+2. Association Product, Association Refer, Reciprocation ยังไม่มี Actual เข้าระบบเลยตลอด 14 วันแรกของรอบ (0 บาททั้ง 3 ช่องทาง เทียบ Target รวม 1,075.19+38.46+67.04 บาท)
+3. Shop Online 1+2 สะสม 3,722.04 บาท ดีกว่า Target 153.26 บาท อย่างมีนัยสำคัญ (+3,568.78 บาท)</t>
         </is>
       </c>
       <c r="B74" s="5" t="n"/>
@@ -3309,9 +3309,9 @@
       <c r="E74" s="5" t="n"/>
       <c r="F74" s="39" t="inlineStr">
         <is>
-          <t>1. แผนก PCRC มีต้นทุนแรงงาน (JRTS) สูงตามโครงสร้างพนักงาน แต่ต้นทุนจริงต่ำกว่าประมาณการที่ตั้งไว้
-2. ข้อมูล Association ยังไม่ถูกบันทึกลงระบบ หรือทีมยังไม่ได้โทรติดตามลูกค้าในช่วง 13 วันที่ผ่านมา
-3. %MA/Revenue สะสม -3.26% ดีกว่า Target -8.15% เนื่องจาก JRTS Actual ต่ำกว่า Target มาก และ Shop Online ทำได้เกินเป้า</t>
+          <t>1. Gross MA สะสม -192,292.35 บาท ดีกว่า Target -482,809.39 บาท อยู่ 290,517.04 บาท (%MA -3.24% vs Target -8.15%) เพราะควบคุมต้นทุน JRTS ได้ต่ำกว่าประมาณการ
+2. ทีมยังไม่ได้บันทึก/โทรติดตามลูกค้าฝั่ง Association และ Reciprocation ในสัปดาห์ 27–28 ที่ผ่านมา
+3. วันที่ 12 กรกฎาคม 2569 (เมื่อวาน) เป็นวันหยุด (Target JRTS = 0) แต่ Actual ยังคงเป็น 0 บาททั้งวัน ต่ำกว่า Target เล็กน้อย (87.75 บาท) ทำให้ %MA วันล่าสุดต่ำกว่า Target</t>
         </is>
       </c>
       <c r="G74" s="5" t="n"/>
@@ -3321,9 +3321,9 @@
       <c r="K74" s="5" t="n"/>
       <c r="L74" s="39" t="inlineStr">
         <is>
-          <t>1. เร่งบันทึก Association Product/Refer ที่ตกค้าง และกระตุ้นทีมโทรติดตามลูกค้าให้ครบ Target 76.80 บาท/วัน
-2. เพิ่มยอด Reciprocation ติดตามลูกค้าซื้อซ้ำ เป้า 6.70 บาท/วัน ซึ่งยังเป็นศูนย์ทุกวัน
-3. วันที่ 11 ก.ค. เป็นวันหยุด ไม่มี Actual — มอบหมายงานติดตามลูกค้าทาง Facebook ให้ปริยณัฐ รุจิชัยวิสิฐ เพื่อปิด Gap</t>
+          <t>1. เร่งบันทึก Association Product/Refer/Reciprocation ที่ยังเป็น 0 บาทให้ทันสัปดาห์ปัจจุบัน (สัปดาห์ 29)
+2. รักษาโมเมนตัม Shop Online ต่อเนื่อง (ปัจจุบันทำได้เกิน Target กว่า 20 เท่า) พร้อมมอบหมายงานเร่งรัดในวันที่ %MA ต่ำกว่า Target
+3. ตรวจสอบการบันทึกข้อมูลวันหยุด (11–12 ก.ค.) ให้ครบถ้วน เพื่อไม่ให้ %MA วันล่าสุดต่ำกว่า Target จากข้อมูลตกหล่น</t>
         </is>
       </c>
       <c r="M74" s="5" t="n"/>
@@ -9540,9 +9540,7 @@
       <c r="X14" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="Y14" s="67" t="n">
-        <v>211702.0397</v>
-      </c>
+      <c r="Y14" s="66" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="66" t="n">
@@ -9621,7 +9619,9 @@
       <c r="X15" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="Y15" s="66" t="n"/>
+      <c r="Y15" s="67" t="n">
+        <v>211702.0397</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -10733,7 +10733,7 @@
         </is>
       </c>
       <c r="C32" s="72" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33">

</xml_diff>